<commit_message>
apos atualizar pagos Asaas
</commit_message>
<xml_diff>
--- a/contas/boleto@manual.com/registros_pedidos.xlsx
+++ b/contas/boleto@manual.com/registros_pedidos.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1143,6 +1143,66 @@
         <v>0</v>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>BLT28</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>46191110000000000004299277852010 2 16070000017690</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>940947595</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>19hr59</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>19/10/2026</t>
+        </is>
+      </c>
+      <c r="F29" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>BLT29</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>46191110000000000004299277876019 9 16070000017690</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>940947774</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>20hr00</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>19/10/2026</t>
+        </is>
+      </c>
+      <c r="F30" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>